<commit_message>
Atualizacao de arquivos - 08/06/2026 19:58:28,55
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1720</v>
+        <v>1717</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3077,7 +3077,7 @@
         <v>2026</v>
       </c>
       <c r="C157">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D157" t="s">
         <v>19</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 10/06/2026  8:55:23,83
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>398</v>
+        <v>383</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3077,7 +3077,7 @@
         <v>2026</v>
       </c>
       <c r="C157">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D157" t="s">
         <v>19</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3111,7 +3111,7 @@
         <v>2026</v>
       </c>
       <c r="C159">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D159" t="s">
         <v>18</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 11/06/2026  1:07:59,63
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1711</v>
+        <v>1695</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 12/06/2026  8:41:12,29
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>380</v>
+        <v>450</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1695</v>
+        <v>1692</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 15/06/2026  8:45:45,12
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>450</v>
+        <v>483</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1692</v>
+        <v>1673</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 16/06/2026  8:57:44,41
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>483</v>
+        <v>573</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1673</v>
+        <v>1683</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/06/2026  8:54:31,93
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>573</v>
+        <v>652</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 18/06/2026  8:44:21,61
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>652</v>
+        <v>661</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1683</v>
+        <v>1674</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 19/06/2026  8:46:31,11
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1674</v>
+        <v>1669</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 22/06/2026  9:20:41,89
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1669</v>
+        <v>1653</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 23/06/2026  8:42:39,08
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1653</v>
+        <v>1651</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>146</v>
+        <v>175</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 24/06/2026  8:49:14,59
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>669</v>
+        <v>657</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1651</v>
+        <v>1654</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 26/06/2026 15:02:59,32
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="23">
   <si>
     <t>Mês</t>
   </si>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>626</v>
+        <v>604</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1651</v>
+        <v>1641</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3077,7 +3077,7 @@
         <v>2026</v>
       </c>
       <c r="C157">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D157" t="s">
         <v>19</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>198</v>
+        <v>249</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3111,29 +3111,12 @@
         <v>2026</v>
       </c>
       <c r="C159">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="D159" t="s">
         <v>18</v>
       </c>
       <c r="E159" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5">
-      <c r="A160" t="s">
-        <v>10</v>
-      </c>
-      <c r="B160">
-        <v>2026</v>
-      </c>
-      <c r="C160">
-        <v>84</v>
-      </c>
-      <c r="D160" t="s">
-        <v>18</v>
-      </c>
-      <c r="E160" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 29/06/2026  8:43:48,49
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1641</v>
+        <v>1631</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3111,7 +3111,7 @@
         <v>2026</v>
       </c>
       <c r="C159">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D159" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 30/06/2026  8:29:54,38
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3043,7 +3043,7 @@
         <v>2026</v>
       </c>
       <c r="C155">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3060,7 +3060,7 @@
         <v>2026</v>
       </c>
       <c r="C156">
-        <v>1631</v>
+        <v>1635</v>
       </c>
       <c r="D156" t="s">
         <v>17</v>
@@ -3094,7 +3094,7 @@
         <v>2026</v>
       </c>
       <c r="C158">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D158" t="s">
         <v>19</v>
@@ -3111,7 +3111,7 @@
         <v>2026</v>
       </c>
       <c r="C159">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D159" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 01/07/2026  8:04:00,34
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="23">
   <si>
     <t>Mês</t>
   </si>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E159"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3120,6 +3120,91 @@
         <v>20</v>
       </c>
     </row>
+    <row r="160" spans="1:5">
+      <c r="A160" t="s">
+        <v>11</v>
+      </c>
+      <c r="B160">
+        <v>2026</v>
+      </c>
+      <c r="C160">
+        <v>601</v>
+      </c>
+      <c r="D160" t="s">
+        <v>17</v>
+      </c>
+      <c r="E160" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5">
+      <c r="A161" t="s">
+        <v>11</v>
+      </c>
+      <c r="B161">
+        <v>2026</v>
+      </c>
+      <c r="C161">
+        <v>1651</v>
+      </c>
+      <c r="D161" t="s">
+        <v>17</v>
+      </c>
+      <c r="E161" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5">
+      <c r="A162" t="s">
+        <v>11</v>
+      </c>
+      <c r="B162">
+        <v>2026</v>
+      </c>
+      <c r="C162">
+        <v>4</v>
+      </c>
+      <c r="D162" t="s">
+        <v>19</v>
+      </c>
+      <c r="E162" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5">
+      <c r="A163" t="s">
+        <v>11</v>
+      </c>
+      <c r="B163">
+        <v>2026</v>
+      </c>
+      <c r="C163">
+        <v>235</v>
+      </c>
+      <c r="D163" t="s">
+        <v>19</v>
+      </c>
+      <c r="E163" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5">
+      <c r="A164" t="s">
+        <v>11</v>
+      </c>
+      <c r="B164">
+        <v>2026</v>
+      </c>
+      <c r="C164">
+        <v>97</v>
+      </c>
+      <c r="D164" t="s">
+        <v>18</v>
+      </c>
+      <c r="E164" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 06/07/2026  9:05:36,66
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>601</v>
+        <v>596</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1651</v>
+        <v>1630</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 07/07/2026  8:56:02,48
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1630</v>
+        <v>1628</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>220</v>
+        <v>274</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 08/07/2026  8:54:56,50
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1628</v>
+        <v>1632</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 09/07/2026  8:45:04,77
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 10/07/2026  8:59:02,27
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>591</v>
+        <v>560</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1634</v>
+        <v>1530</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 13/07/2026  8:52:07,43
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1530</v>
+        <v>1526</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 14/07/2026  9:27:13,62
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>558</v>
+        <v>553</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1526</v>
+        <v>1578</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 15/07/2026  8:59:37,08
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>553</v>
+        <v>758</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1578</v>
+        <v>1582</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3162,7 +3162,7 @@
         <v>2026</v>
       </c>
       <c r="C162">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D162" t="s">
         <v>19</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,7 +3196,7 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 16/07/2026  8:31:12,59
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="23">
   <si>
     <t>Mês</t>
   </si>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>758</v>
+        <v>1010</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3196,12 +3196,29 @@
         <v>2026</v>
       </c>
       <c r="C164">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>
       </c>
       <c r="E164" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5">
+      <c r="A165" t="s">
+        <v>11</v>
+      </c>
+      <c r="B165">
+        <v>2026</v>
+      </c>
+      <c r="C165">
+        <v>82</v>
+      </c>
+      <c r="D165" t="s">
+        <v>18</v>
+      </c>
+      <c r="E165" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/07/2026  8:49:17,95
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1582</v>
+        <v>1587</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 20/07/2026  9:08:53,62
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>1012</v>
+        <v>1003</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1587</v>
+        <v>1584</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>237</v>
+        <v>269</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 21/07/2026  8:35:05,20
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1584</v>
+        <v>1577</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 22/07/2026  9:24:21,30
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1577</v>
+        <v>1571</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 23/07/2026  8:14:45,90
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>990</v>
+        <v>987</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1571</v>
+        <v>1563</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 24/07/2026  8:25:05,29
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1563</v>
+        <v>1572</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 27/07/2026  8:45:31,77
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1572</v>
+        <v>1491</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 28/07/2026  8:10:43,29
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1491</v>
+        <v>1507</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 29/07/2026  8:40:21,52
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>975</v>
+        <v>955</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1507</v>
+        <v>1484</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 30/07/2026  8:39:38,06
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>955</v>
+        <v>934</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1484</v>
+        <v>1477</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 30/07/2026 14:18:00,50
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>934</v>
+        <v>860</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1477</v>
+        <v>1475</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 30/07/2026 18:03:30,75
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>860</v>
+        <v>848</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1475</v>
+        <v>1473</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>
@@ -3213,7 +3213,7 @@
         <v>2026</v>
       </c>
       <c r="C165">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 31/07/2026  8:54:02,85
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -3128,7 +3128,7 @@
         <v>2026</v>
       </c>
       <c r="C160">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="D160" t="s">
         <v>17</v>
@@ -3145,7 +3145,7 @@
         <v>2026</v>
       </c>
       <c r="C161">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="D161" t="s">
         <v>17</v>
@@ -3179,7 +3179,7 @@
         <v>2026</v>
       </c>
       <c r="C163">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D163" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 01/08/2026  8:39:47,09
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="23">
   <si>
     <t>Mês</t>
   </si>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E165"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -3222,6 +3222,108 @@
         <v>20</v>
       </c>
     </row>
+    <row r="166" spans="1:5">
+      <c r="A166" t="s">
+        <v>12</v>
+      </c>
+      <c r="B166">
+        <v>2026</v>
+      </c>
+      <c r="C166">
+        <v>807</v>
+      </c>
+      <c r="D166" t="s">
+        <v>17</v>
+      </c>
+      <c r="E166" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5">
+      <c r="A167" t="s">
+        <v>12</v>
+      </c>
+      <c r="B167">
+        <v>2026</v>
+      </c>
+      <c r="C167">
+        <v>1465</v>
+      </c>
+      <c r="D167" t="s">
+        <v>17</v>
+      </c>
+      <c r="E167" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5">
+      <c r="A168" t="s">
+        <v>12</v>
+      </c>
+      <c r="B168">
+        <v>2026</v>
+      </c>
+      <c r="C168">
+        <v>1</v>
+      </c>
+      <c r="D168" t="s">
+        <v>19</v>
+      </c>
+      <c r="E168" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5">
+      <c r="A169" t="s">
+        <v>12</v>
+      </c>
+      <c r="B169">
+        <v>2026</v>
+      </c>
+      <c r="C169">
+        <v>247</v>
+      </c>
+      <c r="D169" t="s">
+        <v>19</v>
+      </c>
+      <c r="E169" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5">
+      <c r="A170" t="s">
+        <v>12</v>
+      </c>
+      <c r="B170">
+        <v>2026</v>
+      </c>
+      <c r="C170">
+        <v>2</v>
+      </c>
+      <c r="D170" t="s">
+        <v>18</v>
+      </c>
+      <c r="E170" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5">
+      <c r="A171" t="s">
+        <v>12</v>
+      </c>
+      <c r="B171">
+        <v>2026</v>
+      </c>
+      <c r="C171">
+        <v>114</v>
+      </c>
+      <c r="D171" t="s">
+        <v>18</v>
+      </c>
+      <c r="E171" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>